<commit_message>
AJustes en BDD, modelos y campos select2 en pantalla de búsqueda, HTML y js
</commit_message>
<xml_diff>
--- a/SourceFiles/nomenclatura_ATBs.xlsx
+++ b/SourceFiles/nomenclatura_ATBs.xlsx
@@ -87,7 +87,7 @@
     <t xml:space="preserve">    caz = verbose_name="Ceftazidime"</t>
   </si>
   <si>
-    <t xml:space="preserve">CAZ</t>
+    <t xml:space="preserve">CAZ, TAZ*, CZ, TZ</t>
   </si>
   <si>
     <t xml:space="preserve"> help_text="CAZ-ARO:0000060"</t>
@@ -339,7 +339,7 @@
     <t xml:space="preserve">tz = verbose_name="Tazobactam"</t>
   </si>
   <si>
-    <t xml:space="preserve">TZ, TAZ</t>
+    <t xml:space="preserve">TZ, TAZ*</t>
   </si>
   <si>
     <t xml:space="preserve"> help_text="TZ-ARO:0000077"</t>
@@ -544,13 +544,12 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -573,13 +572,17 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <charset val="1"/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFC9211E"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="5">
@@ -591,14 +594,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF2DCDB"/>
-        <bgColor rgb="FFD9D9D9"/>
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor rgb="FFFFFF00"/>
+        <fgColor rgb="FFF2DCDB"/>
+        <bgColor rgb="FFD9D9D9"/>
       </patternFill>
     </fill>
     <fill>
@@ -649,7 +652,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="14">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -662,7 +665,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -670,7 +677,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -690,7 +705,7 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -757,7 +772,7 @@
       <rgbColor rgb="FF339966"/>
       <rgbColor rgb="FF003300"/>
       <rgbColor rgb="FF333300"/>
-      <rgbColor rgb="FF993300"/>
+      <rgbColor rgb="FFC9211E"/>
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FF333399"/>
       <rgbColor rgb="FF333333"/>
@@ -772,7 +787,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D1048576"/>
-  <sheetFormatPr defaultColWidth="10.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.5390625" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="52.85"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="31"/>
@@ -780,7 +795,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="92.14"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -794,7 +809,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
         <v>4</v>
       </c>
@@ -808,7 +823,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
         <v>8</v>
       </c>
@@ -822,7 +837,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
         <v>12</v>
       </c>
@@ -836,7 +851,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
         <v>16</v>
       </c>
@@ -850,11 +865,11 @@
         <v>19</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
         <v>20</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="2" t="s">
         <v>21</v>
       </c>
       <c r="C6" s="0" t="s">
@@ -864,7 +879,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
         <v>24</v>
       </c>
@@ -878,7 +893,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
         <v>28</v>
       </c>
@@ -892,7 +907,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
         <v>32</v>
       </c>
@@ -906,7 +921,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
         <v>36</v>
       </c>
@@ -920,7 +935,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
         <v>40</v>
       </c>
@@ -934,7 +949,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
         <v>44</v>
       </c>
@@ -948,7 +963,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
         <v>48</v>
       </c>
@@ -962,7 +977,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
         <v>52</v>
       </c>
@@ -976,7 +991,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
         <v>56</v>
       </c>
@@ -990,7 +1005,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
         <v>60</v>
       </c>
@@ -1004,53 +1019,53 @@
         <v>63</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="2" t="s">
+    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="B17" s="3" t="s">
+      <c r="B17" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="C17" s="2" t="s">
+      <c r="C17" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="D17" s="2" t="s">
+      <c r="D17" s="3" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="2" t="s">
+    <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="B18" s="3" t="s">
+      <c r="B18" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="C18" s="2" t="s">
+      <c r="C18" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="D18" s="2" t="s">
+      <c r="D18" s="3" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="2" t="s">
+    <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="B19" s="3" t="s">
+      <c r="B19" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="C19" s="2" t="s">
+      <c r="C19" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="D19" s="2" t="s">
+      <c r="D19" s="3" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="0" t="s">
         <v>76</v>
       </c>
-      <c r="B20" s="4" t="s">
+      <c r="B20" s="5" t="s">
         <v>77</v>
       </c>
       <c r="C20" s="0" t="s">
@@ -1060,11 +1075,11 @@
         <v>79</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="0" t="s">
         <v>80</v>
       </c>
-      <c r="B21" s="4" t="s">
+      <c r="B21" s="5" t="s">
         <v>81</v>
       </c>
       <c r="C21" s="0" t="s">
@@ -1074,25 +1089,25 @@
         <v>83</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="2" t="s">
+    <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="B22" s="3" t="s">
+      <c r="B22" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="C22" s="2" t="s">
+      <c r="C22" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="D22" s="2" t="s">
+      <c r="D22" s="3" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="0" t="s">
         <v>88</v>
       </c>
-      <c r="B23" s="4" t="s">
+      <c r="B23" s="5" t="s">
         <v>89</v>
       </c>
       <c r="C23" s="0" t="s">
@@ -1102,11 +1117,11 @@
         <v>91</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="0" t="s">
         <v>92</v>
       </c>
-      <c r="B24" s="4" t="s">
+      <c r="B24" s="5" t="s">
         <v>93</v>
       </c>
       <c r="C24" s="0" t="s">
@@ -1116,11 +1131,11 @@
         <v>95</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="0" t="s">
         <v>96</v>
       </c>
-      <c r="B25" s="4" t="s">
+      <c r="B25" s="5" t="s">
         <v>97</v>
       </c>
       <c r="C25" s="0" t="s">
@@ -1130,11 +1145,11 @@
         <v>99</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="0" t="s">
         <v>100</v>
       </c>
-      <c r="B26" s="4" t="s">
+      <c r="B26" s="5" t="s">
         <v>101</v>
       </c>
       <c r="C26" s="0" t="s">
@@ -1144,17 +1159,17 @@
         <v>103</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="0" t="s">
+    <row r="27" s="6" customFormat="true" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="B27" s="4" t="s">
+      <c r="B27" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="C27" s="0" t="s">
+      <c r="C27" s="6" t="s">
         <v>106</v>
       </c>
-      <c r="D27" s="0" t="s">
+      <c r="D27" s="6" t="s">
         <v>107</v>
       </c>
     </row>
@@ -1223,7 +1238,7 @@
       </c>
     </row>
     <row r="36" customFormat="false" ht="93.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B36" s="5" t="s">
+      <c r="B36" s="8" t="s">
         <v>124</v>
       </c>
     </row>
@@ -1246,253 +1261,253 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="B1:C36"/>
-  <sheetFormatPr defaultColWidth="11.4296875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.4296875" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="6" width="11.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="6" width="27.72"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="7" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="6" width="22.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="6" width="18.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="6" width="20.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="6" width="11.85"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="6" width="27"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="6" width="27.72"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="10" style="6" width="11.43"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="9" width="11.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="9" width="27.72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="10" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="9" width="22.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="9" width="18.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="9" width="20.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="9" width="11.85"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="9" width="27"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="9" width="27.72"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1024" min="10" style="9" width="11.43"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B1" s="8" t="s">
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B1" s="11" t="s">
         <v>125</v>
       </c>
-      <c r="C1" s="9" t="s">
+      <c r="C1" s="12" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="8" t="s">
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B2" s="11" t="s">
         <v>127</v>
       </c>
-      <c r="C2" s="9" t="s">
+      <c r="C2" s="12" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B3" s="8"/>
-      <c r="C3" s="10" t="s">
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B3" s="11"/>
+      <c r="C3" s="13" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B4" s="8" t="s">
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B4" s="11" t="s">
         <v>130</v>
       </c>
-      <c r="C4" s="10" t="s">
+      <c r="C4" s="13" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="8"/>
-      <c r="C5" s="10" t="s">
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B5" s="11"/>
+      <c r="C5" s="13" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="8"/>
-      <c r="C6" s="10" t="s">
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B6" s="11"/>
+      <c r="C6" s="13" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="8"/>
-      <c r="C7" s="10" t="s">
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B7" s="11"/>
+      <c r="C7" s="13" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="8"/>
-      <c r="C8" s="10" t="s">
+    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B8" s="11"/>
+      <c r="C8" s="13" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="8"/>
-      <c r="C9" s="10" t="s">
+    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B9" s="11"/>
+      <c r="C9" s="13" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="8"/>
-      <c r="C10" s="9" t="s">
+    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B10" s="11"/>
+      <c r="C10" s="12" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="8"/>
-      <c r="C11" s="9" t="s">
+    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B11" s="11"/>
+      <c r="C11" s="12" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="8"/>
-      <c r="C12" s="9" t="s">
+    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B12" s="11"/>
+      <c r="C12" s="12" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="8" t="s">
+    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B13" s="11" t="s">
         <v>140</v>
       </c>
-      <c r="C13" s="10" t="s">
+      <c r="C13" s="13" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="8"/>
-      <c r="C14" s="10" t="s">
+    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B14" s="11"/>
+      <c r="C14" s="13" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="8" t="s">
+    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B15" s="11" t="s">
         <v>143</v>
       </c>
-      <c r="C15" s="10" t="s">
+      <c r="C15" s="13" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="8"/>
-      <c r="C16" s="10" t="s">
+    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B16" s="11"/>
+      <c r="C16" s="13" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="8"/>
-      <c r="C17" s="10" t="s">
+    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B17" s="11"/>
+      <c r="C17" s="13" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="8"/>
-      <c r="C18" s="9" t="s">
+    <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B18" s="11"/>
+      <c r="C18" s="12" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="8"/>
-      <c r="C19" s="9" t="s">
+    <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B19" s="11"/>
+      <c r="C19" s="12" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="8"/>
-      <c r="C20" s="9" t="s">
+    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B20" s="11"/>
+      <c r="C20" s="12" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="8" t="s">
+    <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B21" s="11" t="s">
         <v>150</v>
       </c>
-      <c r="C21" s="10" t="s">
+      <c r="C21" s="13" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="8"/>
-      <c r="C22" s="10" t="s">
+    <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B22" s="11"/>
+      <c r="C22" s="13" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B23" s="8"/>
-      <c r="C23" s="9" t="s">
+    <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B23" s="11"/>
+      <c r="C23" s="12" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B24" s="8"/>
-      <c r="C24" s="9" t="s">
+    <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B24" s="11"/>
+      <c r="C24" s="12" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B25" s="8" t="s">
+    <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B25" s="11" t="s">
         <v>155</v>
       </c>
-      <c r="C25" s="10" t="s">
+      <c r="C25" s="13" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B26" s="8"/>
-      <c r="C26" s="9" t="s">
+    <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B26" s="11"/>
+      <c r="C26" s="12" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B27" s="8"/>
-      <c r="C27" s="9" t="s">
+    <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B27" s="11"/>
+      <c r="C27" s="12" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B28" s="8"/>
-      <c r="C28" s="9" t="s">
+    <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B28" s="11"/>
+      <c r="C28" s="12" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B29" s="8" t="s">
+    <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B29" s="11" t="s">
         <v>160</v>
       </c>
-      <c r="C29" s="10" t="s">
+      <c r="C29" s="13" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B30" s="8" t="s">
+    <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B30" s="11" t="s">
         <v>162</v>
       </c>
-      <c r="C30" s="9" t="s">
+      <c r="C30" s="13" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B31" s="8" t="s">
+    <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B31" s="11" t="s">
         <v>164</v>
       </c>
-      <c r="C31" s="9" t="s">
+      <c r="C31" s="12" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B32" s="8"/>
-      <c r="C32" s="9" t="s">
+    <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B32" s="11"/>
+      <c r="C32" s="12" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B33" s="8"/>
-      <c r="C33" s="9" t="s">
+    <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B33" s="11"/>
+      <c r="C33" s="12" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B34" s="8"/>
-      <c r="C34" s="9" t="s">
+    <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B34" s="11"/>
+      <c r="C34" s="12" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B35" s="8"/>
-      <c r="C35" s="9" t="s">
+    <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B35" s="11"/>
+      <c r="C35" s="12" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B36" s="8"/>
-      <c r="C36" s="9" t="s">
+    <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B36" s="11"/>
+      <c r="C36" s="12" t="s">
         <v>170</v>
       </c>
     </row>
@@ -1522,7 +1537,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="10.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.5390625" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>

</xml_diff>